<commit_message>
Updated analysis and tables. Split analysis into a and b
</commit_message>
<xml_diff>
--- a/tables.xlsx
+++ b/tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac.sharepoint.com/sites/r-winterlab/Projects/Colleges - Belonging/colleges_belonging/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\colleges_belonging\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="437" documentId="11_F25DC773A252ABDACC10487339994B0E5ADE58E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EC5E88F-1317-4406-86B1-CBD5FD283E16}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51E5F009-0D81-4681-8BF9-B836FDA0A6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10380" yWindow="2910" windowWidth="16275" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="corr_matrix" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="96">
   <si>
     <t>(Intercept)</t>
   </si>
@@ -240,9 +240,6 @@
     </r>
   </si>
   <si>
-    <t>*** denotes p-value &lt; 0.001</t>
-  </si>
-  <si>
     <t>Est.</t>
   </si>
   <si>
@@ -314,6 +311,141 @@
   <si>
     <t>N = 300</t>
   </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Pre-university identity T1 (1)</t>
+  </si>
+  <si>
+    <t>Wellbeing T1 (2)</t>
+  </si>
+  <si>
+    <t>Identity continuity T2 (3)</t>
+  </si>
+  <si>
+    <t>Identity gain T2 (4)</t>
+  </si>
+  <si>
+    <t>Wellbeing T3 (5)</t>
+  </si>
+  <si>
+    <t>N = 416</t>
+  </si>
+  <si>
+    <r>
+      <t>Note.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> * </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>p</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt; .05, ** </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>p</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt; .01, *** </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>p</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt; .001.</t>
+    </r>
+  </si>
+  <si>
+    <t>0.43***</t>
+  </si>
+  <si>
+    <t>0.26***</t>
+  </si>
+  <si>
+    <t>0.23***</t>
+  </si>
+  <si>
+    <t>0.49***</t>
+  </si>
+  <si>
+    <t>0.27***</t>
+  </si>
+  <si>
+    <t>0.47***</t>
+  </si>
+  <si>
+    <t>0.21***</t>
+  </si>
+  <si>
+    <t>0.28***</t>
+  </si>
+  <si>
+    <t>0.18**</t>
+  </si>
+  <si>
+    <t>ci.lower</t>
+  </si>
+  <si>
+    <t>ci.upper</t>
+  </si>
+  <si>
+    <t>std.all</t>
+  </si>
 </sst>
 </file>
 
@@ -322,7 +454,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,8 +520,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -402,8 +555,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4E5C68"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -440,11 +599,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF0C1F30"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF0C1F30"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF0C1F30"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -483,9 +662,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -509,6 +685,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1724,11 +1913,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{967A851E-614F-4818-A147-967FCF5FBE4F}">
-  <dimension ref="B2:N9"/>
+  <dimension ref="B2:N16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.28515625" customWidth="1"/>
-    <col min="3" max="6" width="5.7109375" customWidth="1"/>
+    <col min="3" max="6" width="7.85546875" style="10" customWidth="1"/>
     <col min="9" max="9" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1738,17 +1927,19 @@
       </c>
     </row>
     <row r="3" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="16"/>
-      <c r="C3" s="17" t="s">
+      <c r="B3" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="16" t="s">
         <v>58</v>
       </c>
       <c r="I3" s="1" t="s">
@@ -1771,7 +1962,7 @@
       </c>
     </row>
     <row r="4" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>53</v>
       </c>
       <c r="C4" s="13"/>
@@ -1783,16 +1974,14 @@
       </c>
     </row>
     <row r="5" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="20">
-        <f>J5</f>
-        <v>0.4</v>
+      <c r="C5" s="19" t="s">
+        <v>84</v>
       </c>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
-      <c r="F5" s="10"/>
       <c r="I5" s="1" t="s">
         <v>51</v>
       </c>
@@ -1801,18 +1990,16 @@
       </c>
     </row>
     <row r="6" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="20">
-        <v>0.23</v>
-      </c>
-      <c r="D6" s="20">
-        <f>K6</f>
-        <v>0.15</v>
-      </c>
-      <c r="E6" s="20"/>
-      <c r="F6" s="10"/>
+      <c r="C6" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="19"/>
       <c r="I6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1824,21 +2011,18 @@
       </c>
     </row>
     <row r="7" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="20">
-        <v>0.4</v>
-      </c>
-      <c r="D7" s="20">
-        <f>K7</f>
-        <v>0.2</v>
-      </c>
-      <c r="E7" s="20">
-        <f>L7</f>
-        <v>0.46</v>
-      </c>
-      <c r="F7" s="10"/>
+      <c r="C7" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>87</v>
+      </c>
       <c r="I7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1853,23 +2037,20 @@
       </c>
     </row>
     <row r="8" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="22">
-        <v>0.26</v>
-      </c>
-      <c r="D8" s="22">
-        <f>K8</f>
-        <v>0.46</v>
-      </c>
-      <c r="E8" s="22">
-        <f>L8</f>
-        <v>0.2</v>
-      </c>
-      <c r="F8" s="22">
-        <f>M8</f>
-        <v>0.28000000000000003</v>
+      <c r="C8" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>91</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>52</v>
@@ -1888,8 +2069,91 @@
       </c>
     </row>
     <row r="9" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="19" t="s">
-        <v>60</v>
+      <c r="B9" s="28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
+      <c r="M10" s="25"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
+      <c r="N11" s="26"/>
+    </row>
+    <row r="12" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I12" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+    </row>
+    <row r="13" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I13" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="J13" s="27">
+        <v>0.43</v>
+      </c>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+    </row>
+    <row r="14" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I14" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="J14" s="27">
+        <v>0.26</v>
+      </c>
+      <c r="K14" s="27">
+        <v>0.18</v>
+      </c>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+    </row>
+    <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I15" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="J15" s="27">
+        <v>0.43</v>
+      </c>
+      <c r="K15" s="27">
+        <v>0.23</v>
+      </c>
+      <c r="L15" s="27">
+        <v>0.49</v>
+      </c>
+      <c r="M15" s="27"/>
+    </row>
+    <row r="16" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I16" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="J16" s="27">
+        <v>0.27</v>
+      </c>
+      <c r="K16" s="27">
+        <v>0.47</v>
+      </c>
+      <c r="L16" s="27">
+        <v>0.21</v>
+      </c>
+      <c r="M16" s="27">
+        <v>0.28000000000000003</v>
       </c>
     </row>
   </sheetData>
@@ -1906,18 +2170,18 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="23" t="s">
-        <v>70</v>
+      <c r="B3" s="22" t="s">
+        <v>69</v>
       </c>
       <c r="K3" s="1"/>
       <c r="L3" t="s">
+        <v>60</v>
+      </c>
+      <c r="M3" t="s">
         <v>61</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>62</v>
-      </c>
-      <c r="N3" t="s">
-        <v>63</v>
       </c>
       <c r="O3" t="s">
         <v>6</v>
@@ -1938,19 +2202,19 @@
         <v>6</v>
       </c>
       <c r="K4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="L4" t="s">
         <v>64</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>65</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>66</v>
       </c>
-      <c r="N4" t="s">
-        <v>67</v>
-      </c>
       <c r="O4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
@@ -1991,7 +2255,7 @@
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6">
         <f>L6</f>
@@ -2063,7 +2327,7 @@
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C8" s="11">
         <f>L8</f>
@@ -2099,7 +2363,7 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2112,7 +2376,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CFCD16B-DAC7-4757-8EE0-599CBD042FE0}">
-  <dimension ref="B2:V22"/>
+  <dimension ref="B2:Y38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.5703125" customWidth="1"/>
@@ -2121,8 +2385,8 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B2" s="25" t="s">
-        <v>75</v>
+      <c r="B2" s="24" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="2:22" x14ac:dyDescent="0.25">
@@ -2172,26 +2436,26 @@
     </row>
     <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>39</v>
       </c>
       <c r="D4" s="13">
         <f>S4</f>
-        <v>3.4000000000000002E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="E4" s="13">
-        <f t="shared" ref="E4:F12" si="0">T4</f>
-        <v>2.5999999999999999E-2</v>
+        <f>T4</f>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="F4" s="13">
-        <f t="shared" si="0"/>
-        <v>1.288</v>
+        <f>U4</f>
+        <v>0.876</v>
       </c>
       <c r="G4" s="9">
         <f>IF(V4&lt;0.001, "&lt; 0.001", ROUND(V4, 3))</f>
-        <v>0.19800000000000001</v>
+        <v>0.38100000000000001</v>
       </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1">
@@ -2210,16 +2474,20 @@
         <v>11</v>
       </c>
       <c r="S4">
-        <v>3.4000000000000002E-2</v>
+        <f>S25</f>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="T4">
-        <v>2.5999999999999999E-2</v>
+        <f t="shared" ref="T4:V4" si="0">T25</f>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="U4">
-        <v>1.288</v>
+        <f t="shared" si="0"/>
+        <v>0.876</v>
       </c>
       <c r="V4">
-        <v>0.19800000000000001</v>
+        <f t="shared" si="0"/>
+        <v>0.38100000000000001</v>
       </c>
     </row>
     <row r="5" spans="2:22" x14ac:dyDescent="0.25">
@@ -2227,20 +2495,20 @@
         <v>41</v>
       </c>
       <c r="D5" s="14">
-        <f t="shared" ref="D5:D6" si="1">S5</f>
-        <v>7.8E-2</v>
+        <f>S5</f>
+        <v>0.08</v>
       </c>
       <c r="E5" s="14">
-        <f t="shared" si="0"/>
-        <v>2.7E-2</v>
+        <f>T5</f>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="F5" s="14">
-        <f t="shared" si="0"/>
-        <v>2.9129999999999998</v>
+        <f>U5</f>
+        <v>2.4540000000000002</v>
       </c>
       <c r="G5" s="10">
-        <f t="shared" ref="G5:G12" si="2">IF(V5&lt;0.001, "&lt; 0.001", ROUND(V5, 3))</f>
-        <v>4.0000000000000001E-3</v>
+        <f>IF(V5&lt;0.001, "&lt; 0.001", ROUND(V5, 3))</f>
+        <v>1.4E-2</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1">
@@ -2259,16 +2527,20 @@
         <v>13</v>
       </c>
       <c r="S5">
-        <v>7.8E-2</v>
+        <f t="shared" ref="S5:V5" si="1">S26</f>
+        <v>0.08</v>
       </c>
       <c r="T5">
-        <v>2.7E-2</v>
+        <f t="shared" si="1"/>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="U5">
-        <v>2.9129999999999998</v>
+        <f t="shared" si="1"/>
+        <v>2.4540000000000002</v>
       </c>
       <c r="V5">
-        <v>4.0000000000000001E-3</v>
+        <f t="shared" si="1"/>
+        <v>1.4E-2</v>
       </c>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.25">
@@ -2276,20 +2548,20 @@
         <v>43</v>
       </c>
       <c r="D6" s="14">
-        <f t="shared" si="1"/>
+        <f>S6</f>
         <v>1.4E-2</v>
       </c>
       <c r="E6" s="14">
-        <f t="shared" si="0"/>
-        <v>3.5000000000000003E-2</v>
+        <f>T6</f>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="F6" s="14">
-        <f t="shared" si="0"/>
-        <v>0.39400000000000002</v>
+        <f>U6</f>
+        <v>0.32700000000000001</v>
       </c>
       <c r="G6" s="10">
-        <f t="shared" si="2"/>
-        <v>0.69399999999999995</v>
+        <f>IF(V6&lt;0.001, "&lt; 0.001", ROUND(V6, 3))</f>
+        <v>0.74399999999999999</v>
       </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1">
@@ -2308,16 +2580,20 @@
         <v>14</v>
       </c>
       <c r="S6">
+        <f t="shared" ref="S6:V6" si="2">S27</f>
         <v>1.4E-2</v>
       </c>
       <c r="T6">
-        <v>3.5000000000000003E-2</v>
+        <f t="shared" si="2"/>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="U6">
-        <v>0.39400000000000002</v>
+        <f t="shared" si="2"/>
+        <v>0.32700000000000001</v>
       </c>
       <c r="V6">
-        <v>0.69399999999999995</v>
+        <f t="shared" si="2"/>
+        <v>0.74399999999999999</v>
       </c>
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.25">
@@ -2326,19 +2602,19 @@
       </c>
       <c r="D7" s="14">
         <f>S7</f>
-        <v>0.188</v>
+        <v>0.192</v>
       </c>
       <c r="E7" s="14">
-        <f t="shared" si="0"/>
-        <v>8.6999999999999994E-2</v>
+        <f>T7</f>
+        <v>9.2999999999999999E-2</v>
       </c>
       <c r="F7" s="14">
-        <f t="shared" si="0"/>
-        <v>2.1539999999999999</v>
+        <f>U7</f>
+        <v>2.0739999999999998</v>
       </c>
       <c r="G7" s="10">
-        <f t="shared" si="2"/>
-        <v>3.1E-2</v>
+        <f>IF(V7&lt;0.001, "&lt; 0.001", ROUND(V7, 3))</f>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="M7" s="1"/>
       <c r="N7" s="1">
@@ -2354,36 +2630,40 @@
         <v>15</v>
       </c>
       <c r="S7">
-        <v>0.188</v>
+        <f t="shared" ref="S7:V7" si="3">S28</f>
+        <v>0.192</v>
       </c>
       <c r="T7">
-        <v>8.6999999999999994E-2</v>
+        <f t="shared" si="3"/>
+        <v>9.2999999999999999E-2</v>
       </c>
       <c r="U7">
-        <v>2.1539999999999999</v>
+        <f t="shared" si="3"/>
+        <v>2.0739999999999998</v>
       </c>
       <c r="V7">
-        <v>3.1E-2</v>
+        <f t="shared" si="3"/>
+        <v>3.7999999999999999E-2</v>
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D8" s="14">
-        <f t="shared" ref="D8:D12" si="3">S8</f>
-        <v>0.44600000000000001</v>
+        <f>S8</f>
+        <v>0.62</v>
       </c>
       <c r="E8" s="14">
-        <f t="shared" si="0"/>
-        <v>6.4000000000000001E-2</v>
+        <f>T8</f>
+        <v>0.11899999999999999</v>
       </c>
       <c r="F8" s="14">
-        <f t="shared" si="0"/>
-        <v>6.9279999999999999</v>
+        <f>U8</f>
+        <v>5.1950000000000003</v>
       </c>
       <c r="G8" s="10" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(V8&lt;0.001, "&lt; 0.001", ROUND(V8, 3))</f>
         <v>&lt; 0.001</v>
       </c>
       <c r="M8" s="1"/>
@@ -2400,39 +2680,43 @@
         <v>51</v>
       </c>
       <c r="S8">
-        <v>0.44600000000000001</v>
+        <f t="shared" ref="S8:V8" si="4">S29</f>
+        <v>0.62</v>
       </c>
       <c r="T8">
-        <v>6.4000000000000001E-2</v>
+        <f t="shared" si="4"/>
+        <v>0.11899999999999999</v>
       </c>
       <c r="U8">
-        <v>6.9279999999999999</v>
+        <f t="shared" si="4"/>
+        <v>5.1950000000000003</v>
       </c>
       <c r="V8">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
         <v>40</v>
       </c>
       <c r="D9" s="14">
-        <f t="shared" si="3"/>
-        <v>0.26900000000000002</v>
+        <f>S9</f>
+        <v>0.315</v>
       </c>
       <c r="E9" s="14">
-        <f t="shared" si="0"/>
-        <v>6.5000000000000002E-2</v>
+        <f>T9</f>
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="F9" s="14">
-        <f t="shared" si="0"/>
-        <v>4.1070000000000002</v>
+        <f>U9</f>
+        <v>4.306</v>
       </c>
       <c r="G9" s="10" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(V9&lt;0.001, "&lt; 0.001", ROUND(V9, 3))</f>
         <v>&lt; 0.001</v>
       </c>
       <c r="M9" s="1"/>
@@ -2452,15 +2736,19 @@
         <v>16</v>
       </c>
       <c r="S9">
-        <v>0.26900000000000002</v>
+        <f t="shared" ref="S9:V9" si="5">S30</f>
+        <v>0.315</v>
       </c>
       <c r="T9">
-        <v>6.5000000000000002E-2</v>
+        <f t="shared" si="5"/>
+        <v>7.2999999999999995E-2</v>
       </c>
       <c r="U9">
-        <v>4.1070000000000002</v>
+        <f t="shared" si="5"/>
+        <v>4.306</v>
       </c>
       <c r="V9">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -2469,20 +2757,20 @@
         <v>46</v>
       </c>
       <c r="D10" s="14">
-        <f t="shared" si="3"/>
-        <v>0.32400000000000001</v>
+        <f>S10</f>
+        <v>0.36</v>
       </c>
       <c r="E10" s="14">
-        <f t="shared" si="0"/>
-        <v>0.192</v>
+        <f>T10</f>
+        <v>0.19900000000000001</v>
       </c>
       <c r="F10" s="14">
-        <f t="shared" si="0"/>
-        <v>1.681</v>
+        <f>U10</f>
+        <v>1.8120000000000001</v>
       </c>
       <c r="G10" s="10">
-        <f t="shared" si="2"/>
-        <v>9.2999999999999999E-2</v>
+        <f>IF(V10&lt;0.001, "&lt; 0.001", ROUND(V10, 3))</f>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="M10" s="1"/>
       <c r="N10" s="1">
@@ -2498,39 +2786,43 @@
         <v>15</v>
       </c>
       <c r="S10">
-        <v>0.32400000000000001</v>
+        <f t="shared" ref="S10:V10" si="6">S31</f>
+        <v>0.36</v>
       </c>
       <c r="T10">
-        <v>0.192</v>
+        <f t="shared" si="6"/>
+        <v>0.19900000000000001</v>
       </c>
       <c r="U10">
-        <v>1.681</v>
+        <f t="shared" si="6"/>
+        <v>1.8120000000000001</v>
       </c>
       <c r="V10">
-        <v>9.2999999999999999E-2</v>
+        <f t="shared" si="6"/>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
       </c>
       <c r="D11" s="14">
-        <f t="shared" si="3"/>
-        <v>0.45700000000000002</v>
+        <f>S11</f>
+        <v>0.52200000000000002</v>
       </c>
       <c r="E11" s="14">
-        <f t="shared" si="0"/>
-        <v>6.3E-2</v>
+        <f>T11</f>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="F11" s="14">
-        <f t="shared" si="0"/>
-        <v>7.2030000000000003</v>
+        <f>U11</f>
+        <v>7.0369999999999999</v>
       </c>
       <c r="G11" s="10" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(V11&lt;0.001, "&lt; 0.001", ROUND(V11, 3))</f>
         <v>&lt; 0.001</v>
       </c>
       <c r="M11" s="1"/>
@@ -2550,15 +2842,19 @@
         <v>17</v>
       </c>
       <c r="S11">
-        <v>0.45700000000000002</v>
+        <f t="shared" ref="S11:V11" si="7">S32</f>
+        <v>0.52200000000000002</v>
       </c>
       <c r="T11">
-        <v>6.3E-2</v>
+        <f t="shared" si="7"/>
+        <v>7.3999999999999996E-2</v>
       </c>
       <c r="U11">
-        <v>7.2030000000000003</v>
+        <f t="shared" si="7"/>
+        <v>7.0369999999999999</v>
       </c>
       <c r="V11">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -2567,20 +2863,20 @@
         <v>46</v>
       </c>
       <c r="D12" s="14">
-        <f t="shared" si="3"/>
-        <v>-2.1000000000000001E-2</v>
+        <f>S12</f>
+        <v>-6.0000000000000001E-3</v>
       </c>
       <c r="E12" s="14">
-        <f t="shared" si="0"/>
-        <v>0.187</v>
+        <f>T12</f>
+        <v>0.183</v>
       </c>
       <c r="F12" s="14">
-        <f t="shared" si="0"/>
-        <v>-0.115</v>
+        <f>U12</f>
+        <v>-0.03</v>
       </c>
       <c r="G12" s="10">
-        <f t="shared" si="2"/>
-        <v>0.90900000000000003</v>
+        <f>IF(V12&lt;0.001, "&lt; 0.001", ROUND(V12, 3))</f>
+        <v>0.97599999999999998</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1">
@@ -2596,23 +2892,27 @@
         <v>15</v>
       </c>
       <c r="S12">
-        <v>-2.1000000000000001E-2</v>
+        <f t="shared" ref="S12:V12" si="8">S33</f>
+        <v>-6.0000000000000001E-3</v>
       </c>
       <c r="T12">
-        <v>0.187</v>
+        <f t="shared" si="8"/>
+        <v>0.183</v>
       </c>
       <c r="U12">
-        <v>-0.115</v>
+        <f t="shared" si="8"/>
+        <v>-0.03</v>
       </c>
       <c r="V12">
-        <v>0.90900000000000003</v>
+        <f t="shared" si="8"/>
+        <v>0.97599999999999998</v>
       </c>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
-      <c r="G13" s="24"/>
+      <c r="G13" s="23"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
@@ -2627,16 +2927,16 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="E14" s="14">
-        <f t="shared" ref="E14:F14" si="4">T18</f>
-        <v>7.0000000000000001E-3</v>
+        <f t="shared" ref="E14:F14" si="9">T18</f>
+        <v>0.01</v>
       </c>
       <c r="F14" s="14">
-        <f t="shared" si="4"/>
-        <v>1.2290000000000001</v>
+        <f t="shared" si="9"/>
+        <v>0.84599999999999997</v>
       </c>
       <c r="G14" s="10">
         <f>IF(V18&lt;0.001, "&lt; 0.001", ROUND(V18, 3))</f>
-        <v>0.219</v>
+        <v>0.39700000000000002</v>
       </c>
       <c r="M14" s="1"/>
     </row>
@@ -2649,35 +2949,35 @@
       </c>
       <c r="D15" s="15">
         <f>S19</f>
-        <v>3.5999999999999997E-2</v>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="E15" s="15">
-        <f t="shared" ref="E15:F15" si="5">T19</f>
-        <v>1.2999999999999999E-2</v>
+        <f t="shared" ref="E15:F15" si="10">T19</f>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="F15" s="15">
-        <f t="shared" si="5"/>
-        <v>2.7010000000000001</v>
+        <f t="shared" si="10"/>
+        <v>2.367</v>
       </c>
       <c r="G15" s="12">
         <f>IF(V19&lt;0.001, "&lt; 0.001", ROUND(V19, 3))</f>
-        <v>7.0000000000000001E-3</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="13:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="13:25" x14ac:dyDescent="0.25">
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="13:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="13:25" x14ac:dyDescent="0.25">
       <c r="M18" s="1"/>
       <c r="N18" s="1">
         <v>19</v>
@@ -2695,19 +2995,23 @@
         <v>18</v>
       </c>
       <c r="S18">
+        <f>S34</f>
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="T18">
-        <v>7.0000000000000001E-3</v>
+        <f t="shared" ref="T18:V18" si="11">T34</f>
+        <v>0.01</v>
       </c>
       <c r="U18">
-        <v>1.2290000000000001</v>
+        <f t="shared" si="11"/>
+        <v>0.84599999999999997</v>
       </c>
       <c r="V18">
-        <v>0.219</v>
-      </c>
-    </row>
-    <row r="19" spans="13:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="11"/>
+        <v>0.39700000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="13:25" x14ac:dyDescent="0.25">
       <c r="M19" s="1"/>
       <c r="N19" s="1">
         <v>20</v>
@@ -2725,19 +3029,23 @@
         <v>21</v>
       </c>
       <c r="S19">
-        <v>3.5999999999999997E-2</v>
+        <f t="shared" ref="S19:V19" si="12">S35</f>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="T19">
-        <v>1.2999999999999999E-2</v>
+        <f t="shared" si="12"/>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="U19">
-        <v>2.7010000000000001</v>
+        <f t="shared" si="12"/>
+        <v>2.367</v>
       </c>
       <c r="V19">
-        <v>7.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="13:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="12"/>
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="13:25" x14ac:dyDescent="0.25">
       <c r="M20" s="1"/>
       <c r="N20" s="1">
         <v>21</v>
@@ -2755,19 +3063,23 @@
         <v>23</v>
       </c>
       <c r="S20">
-        <v>5.8000000000000003E-2</v>
+        <f t="shared" ref="S20:V20" si="13">S36</f>
+        <v>6.4000000000000001E-2</v>
       </c>
       <c r="T20">
-        <v>3.2000000000000001E-2</v>
+        <f t="shared" si="13"/>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="U20">
-        <v>1.8120000000000001</v>
+        <f t="shared" si="13"/>
+        <v>1.5489999999999999</v>
       </c>
       <c r="V20">
-        <v>7.0000000000000007E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="13:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="13"/>
+        <v>0.121</v>
+      </c>
+    </row>
+    <row r="21" spans="13:25" x14ac:dyDescent="0.25">
       <c r="M21" s="1"/>
       <c r="N21" s="1">
         <v>22</v>
@@ -2785,19 +3097,23 @@
         <v>25</v>
       </c>
       <c r="S21">
-        <v>0.154</v>
+        <f t="shared" ref="S21:V21" si="14">S37</f>
+        <v>0.13600000000000001</v>
       </c>
       <c r="T21">
-        <v>0.15</v>
+        <f t="shared" si="14"/>
+        <v>0.183</v>
       </c>
       <c r="U21">
-        <v>1.0269999999999999</v>
+        <f t="shared" si="14"/>
+        <v>0.74299999999999999</v>
       </c>
       <c r="V21">
-        <v>0.30399999999999999</v>
-      </c>
-    </row>
-    <row r="22" spans="13:22" x14ac:dyDescent="0.25">
+        <f t="shared" si="14"/>
+        <v>0.45700000000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="13:25" x14ac:dyDescent="0.25">
       <c r="M22" s="2"/>
       <c r="N22" s="2">
         <v>23</v>
@@ -2815,16 +3131,575 @@
         <v>27</v>
       </c>
       <c r="S22">
-        <v>0.61099999999999999</v>
+        <f t="shared" ref="S22:V22" si="15">S38</f>
+        <v>0.64800000000000002</v>
       </c>
       <c r="T22">
-        <v>0.39500000000000002</v>
+        <f t="shared" si="15"/>
+        <v>0.46700000000000003</v>
       </c>
       <c r="U22">
-        <v>1.546</v>
+        <f t="shared" si="15"/>
+        <v>1.389</v>
       </c>
       <c r="V22">
-        <v>0.122</v>
+        <f t="shared" si="15"/>
+        <v>0.16500000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="O24" t="s">
+        <v>29</v>
+      </c>
+      <c r="P24" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>31</v>
+      </c>
+      <c r="R24" t="s">
+        <v>32</v>
+      </c>
+      <c r="S24" t="s">
+        <v>33</v>
+      </c>
+      <c r="T24" t="s">
+        <v>34</v>
+      </c>
+      <c r="U24" t="s">
+        <v>35</v>
+      </c>
+      <c r="V24" t="s">
+        <v>36</v>
+      </c>
+      <c r="W24" t="s">
+        <v>93</v>
+      </c>
+      <c r="X24" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N25">
+        <v>1</v>
+      </c>
+      <c r="O25" t="s">
+        <v>52</v>
+      </c>
+      <c r="P25" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>10</v>
+      </c>
+      <c r="R25" t="s">
+        <v>11</v>
+      </c>
+      <c r="S25">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="T25">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="U25">
+        <v>0.876</v>
+      </c>
+      <c r="V25">
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="W25">
+        <v>-3.4000000000000002E-2</v>
+      </c>
+      <c r="X25">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="Y25">
+        <v>5.1999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N26">
+        <v>2</v>
+      </c>
+      <c r="O26" t="s">
+        <v>52</v>
+      </c>
+      <c r="P26" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>12</v>
+      </c>
+      <c r="R26" t="s">
+        <v>13</v>
+      </c>
+      <c r="S26">
+        <v>0.08</v>
+      </c>
+      <c r="T26">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="U26">
+        <v>2.4540000000000002</v>
+      </c>
+      <c r="V26">
+        <v>1.4E-2</v>
+      </c>
+      <c r="W26">
+        <v>1.6E-2</v>
+      </c>
+      <c r="X26">
+        <v>0.14299999999999999</v>
+      </c>
+      <c r="Y26">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="27" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N27">
+        <v>3</v>
+      </c>
+      <c r="O27" t="s">
+        <v>52</v>
+      </c>
+      <c r="P27" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>1</v>
+      </c>
+      <c r="R27" t="s">
+        <v>14</v>
+      </c>
+      <c r="S27">
+        <v>1.4E-2</v>
+      </c>
+      <c r="T27">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="U27">
+        <v>0.32700000000000001</v>
+      </c>
+      <c r="V27">
+        <v>0.74399999999999999</v>
+      </c>
+      <c r="W27">
+        <v>-6.9000000000000006E-2</v>
+      </c>
+      <c r="X27">
+        <v>9.7000000000000003E-2</v>
+      </c>
+      <c r="Y27">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N28">
+        <v>4</v>
+      </c>
+      <c r="O28" t="s">
+        <v>52</v>
+      </c>
+      <c r="P28" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>15</v>
+      </c>
+      <c r="S28">
+        <v>0.192</v>
+      </c>
+      <c r="T28">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="U28">
+        <v>2.0739999999999998</v>
+      </c>
+      <c r="V28">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="W28">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="X28">
+        <v>0.374</v>
+      </c>
+      <c r="Y28">
+        <v>9.9000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N29">
+        <v>5</v>
+      </c>
+      <c r="O29" t="s">
+        <v>52</v>
+      </c>
+      <c r="P29" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>51</v>
+      </c>
+      <c r="S29">
+        <v>0.62</v>
+      </c>
+      <c r="T29">
+        <v>0.11899999999999999</v>
+      </c>
+      <c r="U29">
+        <v>5.1950000000000003</v>
+      </c>
+      <c r="V29">
+        <v>0</v>
+      </c>
+      <c r="W29">
+        <v>0.38600000000000001</v>
+      </c>
+      <c r="X29">
+        <v>0.85399999999999998</v>
+      </c>
+      <c r="Y29">
+        <v>0.41299999999999998</v>
+      </c>
+    </row>
+    <row r="30" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N30">
+        <v>6</v>
+      </c>
+      <c r="O30" t="s">
+        <v>10</v>
+      </c>
+      <c r="P30" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>1</v>
+      </c>
+      <c r="R30" t="s">
+        <v>16</v>
+      </c>
+      <c r="S30">
+        <v>0.315</v>
+      </c>
+      <c r="T30">
+        <v>7.2999999999999995E-2</v>
+      </c>
+      <c r="U30">
+        <v>4.306</v>
+      </c>
+      <c r="V30">
+        <v>0</v>
+      </c>
+      <c r="W30">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="X30">
+        <v>0.45900000000000002</v>
+      </c>
+      <c r="Y30">
+        <v>0.25800000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N31">
+        <v>7</v>
+      </c>
+      <c r="O31" t="s">
+        <v>10</v>
+      </c>
+      <c r="P31" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>15</v>
+      </c>
+      <c r="S31">
+        <v>0.36</v>
+      </c>
+      <c r="T31">
+        <v>0.19900000000000001</v>
+      </c>
+      <c r="U31">
+        <v>1.8120000000000001</v>
+      </c>
+      <c r="V31">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="W31">
+        <v>-2.9000000000000001E-2</v>
+      </c>
+      <c r="X31">
+        <v>0.749</v>
+      </c>
+      <c r="Y31">
+        <v>9.8000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="13:25" x14ac:dyDescent="0.25">
+      <c r="N32">
+        <v>8</v>
+      </c>
+      <c r="O32" t="s">
+        <v>12</v>
+      </c>
+      <c r="P32" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>1</v>
+      </c>
+      <c r="R32" t="s">
+        <v>17</v>
+      </c>
+      <c r="S32">
+        <v>0.52200000000000002</v>
+      </c>
+      <c r="T32">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="U32">
+        <v>7.0369999999999999</v>
+      </c>
+      <c r="V32">
+        <v>0</v>
+      </c>
+      <c r="W32">
+        <v>0.377</v>
+      </c>
+      <c r="X32">
+        <v>0.66800000000000004</v>
+      </c>
+      <c r="Y32">
+        <v>0.43099999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="14:25" x14ac:dyDescent="0.25">
+      <c r="N33">
+        <v>9</v>
+      </c>
+      <c r="O33" t="s">
+        <v>12</v>
+      </c>
+      <c r="P33" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>15</v>
+      </c>
+      <c r="S33">
+        <v>-6.0000000000000001E-3</v>
+      </c>
+      <c r="T33">
+        <v>0.183</v>
+      </c>
+      <c r="U33">
+        <v>-0.03</v>
+      </c>
+      <c r="V33">
+        <v>0.97599999999999998</v>
+      </c>
+      <c r="W33">
+        <v>-0.36399999999999999</v>
+      </c>
+      <c r="X33">
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="Y33">
+        <v>-2E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="14:25" x14ac:dyDescent="0.25">
+      <c r="N34">
+        <v>10</v>
+      </c>
+      <c r="O34" t="s">
+        <v>18</v>
+      </c>
+      <c r="P34" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>20</v>
+      </c>
+      <c r="R34" t="s">
+        <v>18</v>
+      </c>
+      <c r="S34">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="T34">
+        <v>0.01</v>
+      </c>
+      <c r="U34">
+        <v>0.84599999999999997</v>
+      </c>
+      <c r="V34">
+        <v>0.39700000000000002</v>
+      </c>
+      <c r="W34">
+        <v>-1.0999999999999999E-2</v>
+      </c>
+      <c r="X34">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="Y34">
+        <v>1.4E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="14:25" x14ac:dyDescent="0.25">
+      <c r="N35">
+        <v>11</v>
+      </c>
+      <c r="O35" t="s">
+        <v>21</v>
+      </c>
+      <c r="P35" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>22</v>
+      </c>
+      <c r="R35" t="s">
+        <v>21</v>
+      </c>
+      <c r="S35">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="T35">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="U35">
+        <v>2.367</v>
+      </c>
+      <c r="V35">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="W35">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="X35">
+        <v>7.5999999999999998E-2</v>
+      </c>
+      <c r="Y35">
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="14:25" x14ac:dyDescent="0.25">
+      <c r="N36">
+        <v>12</v>
+      </c>
+      <c r="O36" t="s">
+        <v>23</v>
+      </c>
+      <c r="P36" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>24</v>
+      </c>
+      <c r="R36" t="s">
+        <v>23</v>
+      </c>
+      <c r="S36">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="T36">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="U36">
+        <v>1.5489999999999999</v>
+      </c>
+      <c r="V36">
+        <v>0.121</v>
+      </c>
+      <c r="W36">
+        <v>-1.7000000000000001E-2</v>
+      </c>
+      <c r="X36">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="Y36">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="37" spans="14:25" x14ac:dyDescent="0.25">
+      <c r="N37">
+        <v>13</v>
+      </c>
+      <c r="O37" t="s">
+        <v>25</v>
+      </c>
+      <c r="P37" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>26</v>
+      </c>
+      <c r="R37" t="s">
+        <v>25</v>
+      </c>
+      <c r="S37">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="T37">
+        <v>0.183</v>
+      </c>
+      <c r="U37">
+        <v>0.74299999999999999</v>
+      </c>
+      <c r="V37">
+        <v>0.45700000000000002</v>
+      </c>
+      <c r="W37">
+        <v>-0.222</v>
+      </c>
+      <c r="X37">
+        <v>0.49399999999999999</v>
+      </c>
+      <c r="Y37">
+        <v>0.13600000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="14:25" x14ac:dyDescent="0.25">
+      <c r="N38">
+        <v>14</v>
+      </c>
+      <c r="O38" t="s">
+        <v>27</v>
+      </c>
+      <c r="P38" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>28</v>
+      </c>
+      <c r="R38" t="s">
+        <v>27</v>
+      </c>
+      <c r="S38">
+        <v>0.64800000000000002</v>
+      </c>
+      <c r="T38">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="U38">
+        <v>1.389</v>
+      </c>
+      <c r="V38">
+        <v>0.16500000000000001</v>
+      </c>
+      <c r="W38">
+        <v>-0.26700000000000002</v>
+      </c>
+      <c r="X38">
+        <v>1.5640000000000001</v>
+      </c>
+      <c r="Y38">
+        <v>0.64800000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -2834,35 +3709,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SetLabel xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a" xsi:nil="true"/>
-    <ProjectType xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c94f73b7-0c39-49d3-8f32-2f3b95265e92" xsi:nil="true"/>
-    <Owner xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Owner>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B5A24ABE3A758346AF3348838206AC79" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3b3bbe3955f66d23d13a189796ab942b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="edfc92ad-21d7-47df-a3ff-01bc0b43552a" xmlns:ns3="c94f73b7-0c39-49d3-8f32-2f3b95265e92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="61febd9fa1ca2566ae14d6f17ff1415e" ns2:_="" ns3:_="">
     <xsd:import namespace="edfc92ad-21d7-47df-a3ff-01bc0b43552a"/>
@@ -3103,10 +3949,50 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SetLabel xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a" xsi:nil="true"/>
+    <ProjectType xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c94f73b7-0c39-49d3-8f32-2f3b95265e92" xsi:nil="true"/>
+    <Owner xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edfc92ad-21d7-47df-a3ff-01bc0b43552a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C452FC83-86A6-42FA-A8D5-AD94829BD962}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1918E80E-4455-465E-ABD0-5E33CB83AF3D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="edfc92ad-21d7-47df-a3ff-01bc0b43552a"/>
+    <ds:schemaRef ds:uri="c94f73b7-0c39-49d3-8f32-2f3b95265e92"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3123,20 +4009,15 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1918E80E-4455-465E-ABD0-5E33CB83AF3D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C452FC83-86A6-42FA-A8D5-AD94829BD962}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="edfc92ad-21d7-47df-a3ff-01bc0b43552a"/>
-    <ds:schemaRef ds:uri="c94f73b7-0c39-49d3-8f32-2f3b95265e92"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d2b2326c-f811-4ccc-abcb-1b955c303c2e}" enabled="1" method="Standard" siteId="{dc781727-710e-4855-bc4c-690266a1b551}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>